<commit_message>
docs: rapikan gaya penulisan dan komentar
</commit_message>
<xml_diff>
--- a/docs/WBS-Helpdesk.xlsx
+++ b/docs/WBS-Helpdesk.xlsx
@@ -843,7 +843,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Aplikasi Helpdesk (end-to-end)</t>
+          <t>Aplikasi Helpdesk (widget, web, mobile)</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -949,7 +949,7 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>BPMN swimlane end-to-end</t>
+          <t>BPMN swimlane alur tiket</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -1060,7 +1060,7 @@
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>13+ tabel: users, customers, tickets, ticket_messages, ticket_events, attachments, categories, canned_responses, kb_articles, devices, notifications, ai_logs.</t>
+          <t>12 tabel: users, categories, tickets, ticket_messages, message_receipts, ticket_events, attachments, canned_responses, kb_articles, devices, notifications, ai_logs.</t>
         </is>
       </c>
       <c r="E9" s="10" t="inlineStr">
@@ -3869,7 +3869,7 @@
       </c>
       <c r="D62" s="12" t="inlineStr">
         <is>
-          <t>Keystore release, build APK, uji install di perangkat/emulator.</t>
+          <t>Build APK release dengan debug signing untuk demo, lalu uji install di emulator/perangkat.</t>
         </is>
       </c>
       <c r="E62" s="10" t="inlineStr">
@@ -3975,7 +3975,7 @@
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Pengujian end-to-end, perbaikan, dokumentasi, dan paket deliverable.</t>
+          <t>Pengujian alur utama, perbaikan, dokumentasi, dan paket deliverable.</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
@@ -4023,7 +4023,7 @@
       </c>
       <c r="C65" s="11" t="inlineStr">
         <is>
-          <t>E2E widget ↔ web ↔ mobile</t>
+          <t>Uji alur widget ↔ web ↔ mobile</t>
         </is>
       </c>
       <c r="D65" s="12" t="inlineStr">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="C7" s="39" t="inlineStr">
         <is>
-          <t>E2E lintas kanal, uji putus-sambung, bug fixing, README &amp; screenshot, export PDF/XLSX, publish repo publik, kirim email.</t>
+          <t>Uji alur lintas kanal, uji putus-sambung, bug fixing, README &amp; screenshot, export PDF/XLSX, publish repo publik, kirim email.</t>
         </is>
       </c>
       <c r="D7" s="39" t="inlineStr">
@@ -5256,7 +5256,7 @@
       </c>
       <c r="F7" s="39" t="inlineStr">
         <is>
-          <t>Email terkirim sebelum 23:59 WIB (target 12.00 WIB).</t>
+          <t>Email terkirim sebelum 23:59 WIB (target 09.00 WIB).</t>
         </is>
       </c>
     </row>

</xml_diff>